<commit_message>
Recomendacoes: M. Moreno (Paredes) e Marcelino Moreno fora; Reinaldo (Chaves) no lugar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EuPBN7B2QoMn8WDwKax4KN
</commit_message>
<xml_diff>
--- a/Santa Cruz V2/listas/bola_parada_especialistas.xlsx
+++ b/Santa Cruz V2/listas/bola_parada_especialistas.xlsx
@@ -1070,12 +1070,12 @@
     <t>Evander</t>
   </si>
   <si>
+    <t>J. Bartolo</t>
+  </si>
+  <si>
     <t>Arthur Rezende</t>
   </si>
   <si>
-    <t>J. Bartolo</t>
-  </si>
-  <si>
     <t>Valdívia</t>
   </si>
   <si>
@@ -1088,12 +1088,12 @@
     <t>Everton Bala</t>
   </si>
   <si>
+    <t>Thauan Lara</t>
+  </si>
+  <si>
     <t>Gabriel Honório</t>
   </si>
   <si>
-    <t>Thauan Lara</t>
-  </si>
-  <si>
     <t>Gustavo Sauer</t>
   </si>
   <si>
@@ -1145,12 +1145,12 @@
     <t>Cincinnati</t>
   </si>
   <si>
+    <t>Asteras Tripolis</t>
+  </si>
+  <si>
     <t>Muharraq</t>
   </si>
   <si>
-    <t>Asteras Tripolis</t>
-  </si>
-  <si>
     <t>Jeonnam Dragons</t>
   </si>
   <si>
@@ -1280,10 +1280,10 @@
     <t>Wesley</t>
   </si>
   <si>
+    <t>Iago Maidana</t>
+  </si>
+  <si>
     <t>Gastón Valles</t>
-  </si>
-  <si>
-    <t>Iago Maidana</t>
   </si>
   <si>
     <t>Mateus Sarará</t>
@@ -10424,10 +10424,10 @@
     </row>
     <row r="10" spans="1:16">
       <c r="A10" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
         <v>349</v>
@@ -10436,45 +10436,48 @@
         <v>374</v>
       </c>
       <c r="E10">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F10">
-        <v>1839</v>
+        <v>2529</v>
+      </c>
+      <c r="G10" t="s">
+        <v>389</v>
       </c>
       <c r="H10">
-        <v>500000</v>
+        <v>600000</v>
       </c>
       <c r="I10" t="s">
-        <v>82</v>
+        <v>180</v>
       </c>
       <c r="J10">
         <v>92.59999999999999</v>
       </c>
       <c r="K10">
-        <v>56</v>
+        <v>104</v>
       </c>
       <c r="L10">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="M10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N10">
-        <v>22.2</v>
+        <v>37.5</v>
       </c>
       <c r="O10">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="P10">
-        <v>38.1</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="11" spans="1:16">
       <c r="A11" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="C11" t="s">
         <v>350</v>
@@ -10483,40 +10486,37 @@
         <v>375</v>
       </c>
       <c r="E11">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F11">
-        <v>2529</v>
-      </c>
-      <c r="G11" t="s">
-        <v>389</v>
+        <v>1839</v>
       </c>
       <c r="H11">
-        <v>600000</v>
+        <v>500000</v>
       </c>
       <c r="I11" t="s">
-        <v>180</v>
+        <v>82</v>
       </c>
       <c r="J11">
         <v>92.59999999999999</v>
       </c>
       <c r="K11">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="L11">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="M11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N11">
-        <v>37.5</v>
+        <v>22.2</v>
       </c>
       <c r="O11">
-        <v>0.21</v>
+        <v>0.16</v>
       </c>
       <c r="P11">
-        <v>28.6</v>
+        <v>38.1</v>
       </c>
     </row>
     <row r="12" spans="1:16">
@@ -10721,7 +10721,7 @@
     </row>
     <row r="16" spans="1:16">
       <c r="A16" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="B16" t="s">
         <v>23</v>
@@ -10730,16 +10730,19 @@
         <v>355</v>
       </c>
       <c r="D16" t="s">
-        <v>380</v>
+        <v>371</v>
       </c>
       <c r="E16">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="F16">
-        <v>1443</v>
+        <v>1202</v>
+      </c>
+      <c r="G16" t="s">
+        <v>76</v>
       </c>
       <c r="H16">
-        <v>175000</v>
+        <v>0</v>
       </c>
       <c r="I16" t="s">
         <v>82</v>
@@ -10748,27 +10751,27 @@
         <v>91.7</v>
       </c>
       <c r="K16">
-        <v>44</v>
+        <v>59</v>
       </c>
       <c r="L16">
-        <v>18</v>
+        <v>42</v>
       </c>
       <c r="M16">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="N16">
-        <v>57.1</v>
+        <v>66.7</v>
       </c>
       <c r="O16">
-        <v>0.17</v>
+        <v>0.29</v>
       </c>
       <c r="P16">
-        <v>34.9</v>
+        <v>21.7</v>
       </c>
     </row>
     <row r="17" spans="1:16">
       <c r="A17" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
       <c r="B17" t="s">
         <v>23</v>
@@ -10777,19 +10780,16 @@
         <v>356</v>
       </c>
       <c r="D17" t="s">
-        <v>371</v>
+        <v>380</v>
       </c>
       <c r="E17">
-        <v>22</v>
+        <v>30</v>
       </c>
       <c r="F17">
-        <v>1202</v>
-      </c>
-      <c r="G17" t="s">
-        <v>76</v>
+        <v>1443</v>
       </c>
       <c r="H17">
-        <v>0</v>
+        <v>175000</v>
       </c>
       <c r="I17" t="s">
         <v>82</v>
@@ -10798,22 +10798,22 @@
         <v>91.7</v>
       </c>
       <c r="K17">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="L17">
-        <v>42</v>
+        <v>18</v>
       </c>
       <c r="M17">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="N17">
-        <v>66.7</v>
+        <v>57.1</v>
       </c>
       <c r="O17">
-        <v>0.29</v>
+        <v>0.17</v>
       </c>
       <c r="P17">
-        <v>21.7</v>
+        <v>34.9</v>
       </c>
     </row>
     <row r="18" spans="1:16">
@@ -12341,96 +12341,96 @@
     </row>
     <row r="24" spans="1:15">
       <c r="A24" t="s">
-        <v>396</v>
+        <v>337</v>
       </c>
       <c r="B24" t="s">
-        <v>29</v>
+        <v>100</v>
       </c>
       <c r="C24" t="s">
         <v>419</v>
       </c>
       <c r="D24" t="s">
-        <v>439</v>
+        <v>432</v>
       </c>
       <c r="E24">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="F24">
-        <v>1572</v>
+        <v>1533</v>
       </c>
       <c r="G24" t="s">
-        <v>178</v>
+        <v>73</v>
       </c>
       <c r="H24">
-        <v>0</v>
+        <v>1200000</v>
       </c>
       <c r="I24" t="s">
-        <v>276</v>
+        <v>82</v>
       </c>
       <c r="J24">
         <v>85.09999999999999</v>
       </c>
       <c r="K24">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L24">
-        <v>0.11</v>
+        <v>0.06</v>
       </c>
       <c r="M24">
-        <v>7.27</v>
+        <v>4.99</v>
       </c>
       <c r="N24">
-        <v>39.4</v>
+        <v>58.8</v>
       </c>
       <c r="O24">
-        <v>192</v>
+        <v>195</v>
       </c>
     </row>
     <row r="25" spans="1:15">
       <c r="A25" t="s">
-        <v>337</v>
+        <v>396</v>
       </c>
       <c r="B25" t="s">
-        <v>100</v>
+        <v>29</v>
       </c>
       <c r="C25" t="s">
         <v>420</v>
       </c>
       <c r="D25" t="s">
-        <v>432</v>
+        <v>439</v>
       </c>
       <c r="E25">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F25">
-        <v>1533</v>
+        <v>1572</v>
       </c>
       <c r="G25" t="s">
-        <v>73</v>
+        <v>178</v>
       </c>
       <c r="H25">
-        <v>1200000</v>
+        <v>0</v>
       </c>
       <c r="I25" t="s">
-        <v>82</v>
+        <v>276</v>
       </c>
       <c r="J25">
         <v>85.09999999999999</v>
       </c>
       <c r="K25">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="L25">
-        <v>0.06</v>
+        <v>0.11</v>
       </c>
       <c r="M25">
-        <v>4.99</v>
+        <v>7.27</v>
       </c>
       <c r="N25">
-        <v>58.8</v>
+        <v>39.4</v>
       </c>
       <c r="O25">
-        <v>195</v>
+        <v>192</v>
       </c>
     </row>
     <row r="26" spans="1:15">

</xml_diff>

<commit_message>
Dodo fora (foi para a Coreia): Frizzo vira o MEI no 1; Boschilia como opcao; listas regeradas
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EuPBN7B2QoMn8WDwKax4KN
</commit_message>
<xml_diff>
--- a/Santa Cruz V2/listas/bola_parada_especialistas.xlsx
+++ b/Santa Cruz V2/listas/bola_parada_especialistas.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1313" uniqueCount="442">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1312" uniqueCount="442">
   <si>
     <t>liga</t>
   </si>
@@ -104,12 +104,12 @@
     <t>EE</t>
   </si>
   <si>
+    <t>LD</t>
+  </si>
+  <si>
     <t>MEI</t>
   </si>
   <si>
-    <t>LD</t>
-  </si>
-  <si>
     <t>CA</t>
   </si>
   <si>
@@ -128,9 +128,6 @@
     <t>Iago Teles</t>
   </si>
   <si>
-    <t>Dodô</t>
-  </si>
-  <si>
     <t>Pepê</t>
   </si>
   <si>
@@ -173,12 +170,12 @@
     <t>Gegé</t>
   </si>
   <si>
+    <t>Mikael Doka</t>
+  </si>
+  <si>
     <t>Jean Lucas</t>
   </si>
   <si>
-    <t>Mikael Doka</t>
-  </si>
-  <si>
     <t>Dadá Belmonte</t>
   </si>
   <si>
@@ -191,6 +188,9 @@
     <t>Pará</t>
   </si>
   <si>
+    <t>Wesley Pinheiro</t>
+  </si>
+  <si>
     <t>Criciúma</t>
   </si>
   <si>
@@ -203,205 +203,205 @@
     <t>Londrina</t>
   </si>
   <si>
+    <t>Cuiabá</t>
+  </si>
+  <si>
+    <t>América-MG</t>
+  </si>
+  <si>
+    <t>Athletic</t>
+  </si>
+  <si>
+    <t>Sport</t>
+  </si>
+  <si>
+    <t>Fortaleza</t>
+  </si>
+  <si>
+    <t>Operário-PR</t>
+  </si>
+  <si>
+    <t>Avaí</t>
+  </si>
+  <si>
+    <t>Ceará</t>
+  </si>
+  <si>
+    <t>Juventude</t>
+  </si>
+  <si>
+    <t>CRB</t>
+  </si>
+  <si>
+    <t>Goiás</t>
+  </si>
+  <si>
+    <t>Atlético-GO</t>
+  </si>
+  <si>
+    <t>2026-12-31</t>
+  </si>
+  <si>
+    <t>2026-11-30</t>
+  </si>
+  <si>
+    <t>2027-12-31</t>
+  </si>
+  <si>
+    <t>2027-06-30</t>
+  </si>
+  <si>
+    <t>2029-07-31</t>
+  </si>
+  <si>
+    <t>2027-11-30</t>
+  </si>
+  <si>
+    <t>2028-12-31</t>
+  </si>
+  <si>
+    <t>2027-03-31</t>
+  </si>
+  <si>
+    <t>Venezuela</t>
+  </si>
+  <si>
+    <t>Brazil</t>
+  </si>
+  <si>
+    <t>Paraguay</t>
+  </si>
+  <si>
+    <t>Ecuador</t>
+  </si>
+  <si>
+    <t>Brazil, Italy</t>
+  </si>
+  <si>
+    <t>Brazil, Germany</t>
+  </si>
+  <si>
+    <t>indice_finalizador</t>
+  </si>
+  <si>
+    <t>Head goals</t>
+  </si>
+  <si>
+    <t>Head goals per 90</t>
+  </si>
+  <si>
+    <t>Aerial duels per 90</t>
+  </si>
+  <si>
+    <t>Aerial duels won, %</t>
+  </si>
+  <si>
+    <t>Height</t>
+  </si>
+  <si>
+    <t>finalizador_2025</t>
+  </si>
+  <si>
+    <t>gols_cabeca_2025</t>
+  </si>
+  <si>
+    <t>gols_bp_2026</t>
+  </si>
+  <si>
+    <t>gols_bp_3t</t>
+  </si>
+  <si>
+    <t>gols_bp_cabeca_3t</t>
+  </si>
+  <si>
+    <t>xg_bp_3t</t>
+  </si>
+  <si>
+    <t>ZE</t>
+  </si>
+  <si>
+    <t>ZD</t>
+  </si>
+  <si>
+    <t>Luiz Otávio</t>
+  </si>
+  <si>
+    <t>Vilar</t>
+  </si>
+  <si>
+    <t>Alisson Safira</t>
+  </si>
+  <si>
+    <t>Matheus Bianqui</t>
+  </si>
+  <si>
+    <t>Yago Lincoln</t>
+  </si>
+  <si>
+    <t>Dudu</t>
+  </si>
+  <si>
+    <t>Messias</t>
+  </si>
+  <si>
+    <t>Gabriel Pinheiro</t>
+  </si>
+  <si>
+    <t>Kadu</t>
+  </si>
+  <si>
+    <t>Mikael</t>
+  </si>
+  <si>
+    <t>Paulo Vitor</t>
+  </si>
+  <si>
+    <t>Everton Morelli</t>
+  </si>
+  <si>
+    <t>Léo Índio</t>
+  </si>
+  <si>
+    <t>Benevenuto</t>
+  </si>
+  <si>
+    <t>Júlio César</t>
+  </si>
+  <si>
+    <t>J. Miritello</t>
+  </si>
+  <si>
+    <t>André Luiz</t>
+  </si>
+  <si>
+    <t>Léo Gomes</t>
+  </si>
+  <si>
+    <t>Perotti</t>
+  </si>
+  <si>
+    <t>Bruno José</t>
+  </si>
+  <si>
+    <t>Gustavo Coutinho</t>
+  </si>
+  <si>
+    <t>G. Mastriani</t>
+  </si>
+  <si>
+    <t>Kauan Cristtyan</t>
+  </si>
+  <si>
+    <t>Willean Lepo</t>
+  </si>
+  <si>
+    <t>Novorizontino</t>
+  </si>
+  <si>
+    <t>Vila Nova</t>
+  </si>
+  <si>
     <t>Náutico</t>
-  </si>
-  <si>
-    <t>Cuiabá</t>
-  </si>
-  <si>
-    <t>América-MG</t>
-  </si>
-  <si>
-    <t>Athletic</t>
-  </si>
-  <si>
-    <t>Sport</t>
-  </si>
-  <si>
-    <t>Fortaleza</t>
-  </si>
-  <si>
-    <t>Operário-PR</t>
-  </si>
-  <si>
-    <t>Avaí</t>
-  </si>
-  <si>
-    <t>Ceará</t>
-  </si>
-  <si>
-    <t>Juventude</t>
-  </si>
-  <si>
-    <t>CRB</t>
-  </si>
-  <si>
-    <t>Goiás</t>
-  </si>
-  <si>
-    <t>Atlético-GO</t>
-  </si>
-  <si>
-    <t>2026-12-31</t>
-  </si>
-  <si>
-    <t>2026-11-30</t>
-  </si>
-  <si>
-    <t>2027-12-31</t>
-  </si>
-  <si>
-    <t>2027-06-30</t>
-  </si>
-  <si>
-    <t>2029-07-31</t>
-  </si>
-  <si>
-    <t>2027-11-30</t>
-  </si>
-  <si>
-    <t>2028-12-31</t>
-  </si>
-  <si>
-    <t>2027-03-31</t>
-  </si>
-  <si>
-    <t>Venezuela</t>
-  </si>
-  <si>
-    <t>Brazil</t>
-  </si>
-  <si>
-    <t>Paraguay</t>
-  </si>
-  <si>
-    <t>Ecuador</t>
-  </si>
-  <si>
-    <t>Brazil, Italy</t>
-  </si>
-  <si>
-    <t>Brazil, Germany</t>
-  </si>
-  <si>
-    <t>indice_finalizador</t>
-  </si>
-  <si>
-    <t>Head goals</t>
-  </si>
-  <si>
-    <t>Head goals per 90</t>
-  </si>
-  <si>
-    <t>Aerial duels per 90</t>
-  </si>
-  <si>
-    <t>Aerial duels won, %</t>
-  </si>
-  <si>
-    <t>Height</t>
-  </si>
-  <si>
-    <t>finalizador_2025</t>
-  </si>
-  <si>
-    <t>gols_cabeca_2025</t>
-  </si>
-  <si>
-    <t>gols_bp_2026</t>
-  </si>
-  <si>
-    <t>gols_bp_3t</t>
-  </si>
-  <si>
-    <t>gols_bp_cabeca_3t</t>
-  </si>
-  <si>
-    <t>xg_bp_3t</t>
-  </si>
-  <si>
-    <t>ZE</t>
-  </si>
-  <si>
-    <t>ZD</t>
-  </si>
-  <si>
-    <t>Luiz Otávio</t>
-  </si>
-  <si>
-    <t>Vilar</t>
-  </si>
-  <si>
-    <t>Alisson Safira</t>
-  </si>
-  <si>
-    <t>Matheus Bianqui</t>
-  </si>
-  <si>
-    <t>Yago Lincoln</t>
-  </si>
-  <si>
-    <t>Dudu</t>
-  </si>
-  <si>
-    <t>Messias</t>
-  </si>
-  <si>
-    <t>Gabriel Pinheiro</t>
-  </si>
-  <si>
-    <t>Kadu</t>
-  </si>
-  <si>
-    <t>Mikael</t>
-  </si>
-  <si>
-    <t>Paulo Vitor</t>
-  </si>
-  <si>
-    <t>Everton Morelli</t>
-  </si>
-  <si>
-    <t>Léo Índio</t>
-  </si>
-  <si>
-    <t>Benevenuto</t>
-  </si>
-  <si>
-    <t>Júlio César</t>
-  </si>
-  <si>
-    <t>J. Miritello</t>
-  </si>
-  <si>
-    <t>André Luiz</t>
-  </si>
-  <si>
-    <t>Léo Gomes</t>
-  </si>
-  <si>
-    <t>Perotti</t>
-  </si>
-  <si>
-    <t>Bruno José</t>
-  </si>
-  <si>
-    <t>Gustavo Coutinho</t>
-  </si>
-  <si>
-    <t>G. Mastriani</t>
-  </si>
-  <si>
-    <t>Kauan Cristtyan</t>
-  </si>
-  <si>
-    <t>Willean Lepo</t>
-  </si>
-  <si>
-    <t>Novorizontino</t>
-  </si>
-  <si>
-    <t>Vila Nova</t>
   </si>
   <si>
     <t>Ponte Preta</t>
@@ -1795,13 +1795,13 @@
         <v>1477</v>
       </c>
       <c r="G2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H2">
         <v>800000</v>
       </c>
       <c r="I2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J2">
         <v>96.5</v>
@@ -1857,13 +1857,13 @@
         <v>1987</v>
       </c>
       <c r="G3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H3">
         <v>600000</v>
       </c>
       <c r="I3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J3">
         <v>95.90000000000001</v>
@@ -1925,10 +1925,10 @@
         <v>2106</v>
       </c>
       <c r="G4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J4">
         <v>95.2</v>
@@ -1984,10 +1984,10 @@
         <v>1103</v>
       </c>
       <c r="G5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="I5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J5">
         <v>92</v>
@@ -2028,7 +2028,7 @@
         <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
         <v>35</v>
@@ -2037,55 +2037,49 @@
         <v>60</v>
       </c>
       <c r="E6">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F6">
-        <v>1516</v>
+        <v>1571</v>
       </c>
       <c r="G6" t="s">
         <v>74</v>
       </c>
       <c r="I6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J6">
-        <v>91.7</v>
+        <v>91.2</v>
       </c>
       <c r="K6">
-        <v>98</v>
+        <v>65</v>
       </c>
       <c r="L6">
-        <v>42</v>
+        <v>28</v>
       </c>
       <c r="M6">
-        <v>9</v>
+        <v>3</v>
       </c>
       <c r="N6">
-        <v>44.4</v>
+        <v>33.3</v>
       </c>
       <c r="O6">
-        <v>0.34</v>
+        <v>0.13</v>
       </c>
       <c r="P6">
-        <v>22.6</v>
-      </c>
-      <c r="Q6">
-        <v>95.2</v>
-      </c>
-      <c r="R6">
-        <v>76</v>
+        <v>35.7</v>
       </c>
       <c r="S6">
+        <v>3</v>
+      </c>
+      <c r="T6">
+        <v>3</v>
+      </c>
+      <c r="U6">
         <v>2</v>
       </c>
-      <c r="T6">
-        <v>5</v>
-      </c>
-      <c r="U6">
-        <v>4</v>
-      </c>
       <c r="V6">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="7" spans="1:22">
@@ -2093,7 +2087,7 @@
         <v>22</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
         <v>36</v>
@@ -2102,43 +2096,43 @@
         <v>61</v>
       </c>
       <c r="E7">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="F7">
-        <v>1571</v>
+        <v>1303</v>
       </c>
       <c r="G7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="I7" t="s">
         <v>82</v>
       </c>
       <c r="J7">
-        <v>91.2</v>
+        <v>90.40000000000001</v>
       </c>
       <c r="K7">
-        <v>65</v>
+        <v>31</v>
       </c>
       <c r="L7">
-        <v>28</v>
+        <v>12</v>
       </c>
       <c r="M7">
         <v>3</v>
       </c>
       <c r="N7">
-        <v>33.3</v>
+        <v>66.7</v>
       </c>
       <c r="O7">
-        <v>0.13</v>
+        <v>0.25</v>
       </c>
       <c r="P7">
-        <v>35.7</v>
+        <v>38.7</v>
       </c>
       <c r="S7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U7">
         <v>2</v>
@@ -2152,7 +2146,7 @@
         <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="C8" t="s">
         <v>37</v>
@@ -2164,43 +2158,43 @@
         <v>23</v>
       </c>
       <c r="F8">
-        <v>1303</v>
+        <v>1011</v>
       </c>
       <c r="G8" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I8" t="s">
         <v>83</v>
       </c>
       <c r="J8">
-        <v>90.40000000000001</v>
+        <v>90.2</v>
       </c>
       <c r="K8">
-        <v>31</v>
+        <v>22</v>
       </c>
       <c r="L8">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="M8">
         <v>3</v>
       </c>
       <c r="N8">
-        <v>66.7</v>
+        <v>100</v>
       </c>
       <c r="O8">
-        <v>0.25</v>
+        <v>0.17</v>
       </c>
       <c r="P8">
-        <v>38.7</v>
+        <v>33.3</v>
       </c>
       <c r="S8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V8">
         <v>0</v>
@@ -2211,7 +2205,7 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
         <v>38</v>
@@ -2220,43 +2214,43 @@
         <v>63</v>
       </c>
       <c r="E9">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="F9">
-        <v>1011</v>
+        <v>1991</v>
       </c>
       <c r="G9" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="I9" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="J9">
-        <v>90.2</v>
+        <v>90.09999999999999</v>
       </c>
       <c r="K9">
-        <v>22</v>
+        <v>50</v>
       </c>
       <c r="L9">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="M9">
         <v>3</v>
       </c>
       <c r="N9">
-        <v>100</v>
+        <v>33.3</v>
       </c>
       <c r="O9">
-        <v>0.17</v>
+        <v>0.22</v>
       </c>
       <c r="P9">
-        <v>33.3</v>
+        <v>41.8</v>
       </c>
       <c r="S9">
         <v>0</v>
       </c>
       <c r="T9">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U9">
         <v>0</v>
@@ -2270,7 +2264,7 @@
         <v>22</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="C10" t="s">
         <v>39</v>
@@ -2279,49 +2273,55 @@
         <v>64</v>
       </c>
       <c r="E10">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="F10">
-        <v>1991</v>
+        <v>1838</v>
       </c>
       <c r="G10" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="I10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J10">
-        <v>90.09999999999999</v>
+        <v>89.5</v>
       </c>
       <c r="K10">
-        <v>50</v>
+        <v>67</v>
       </c>
       <c r="L10">
-        <v>18</v>
+        <v>38</v>
       </c>
       <c r="M10">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="N10">
-        <v>33.3</v>
+        <v>12.5</v>
       </c>
       <c r="O10">
         <v>0.22</v>
       </c>
       <c r="P10">
-        <v>41.8</v>
+        <v>23</v>
+      </c>
+      <c r="Q10">
+        <v>90.59999999999999</v>
+      </c>
+      <c r="R10">
+        <v>67</v>
       </c>
       <c r="S10">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T10">
+        <v>1</v>
+      </c>
+      <c r="U10">
+        <v>1</v>
+      </c>
+      <c r="V10">
         <v>2</v>
-      </c>
-      <c r="U10">
-        <v>0</v>
-      </c>
-      <c r="V10">
-        <v>0</v>
       </c>
     </row>
     <row r="11" spans="1:22">
@@ -2338,55 +2338,55 @@
         <v>65</v>
       </c>
       <c r="E11">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="F11">
-        <v>1838</v>
+        <v>2396</v>
       </c>
       <c r="G11" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="I11" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="J11">
-        <v>89.5</v>
+        <v>89</v>
       </c>
       <c r="K11">
-        <v>67</v>
+        <v>80</v>
       </c>
       <c r="L11">
-        <v>38</v>
+        <v>63</v>
       </c>
       <c r="M11">
-        <v>8</v>
+        <v>17</v>
       </c>
       <c r="N11">
-        <v>12.5</v>
+        <v>47.1</v>
       </c>
       <c r="O11">
-        <v>0.22</v>
+        <v>0.13</v>
       </c>
       <c r="P11">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="Q11">
-        <v>90.59999999999999</v>
+        <v>96.59999999999999</v>
       </c>
       <c r="R11">
-        <v>67</v>
+        <v>102</v>
       </c>
       <c r="S11">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T11">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="U11">
         <v>1</v>
       </c>
       <c r="V11">
-        <v>2</v>
+        <v>5</v>
       </c>
     </row>
     <row r="12" spans="1:22">
@@ -2394,7 +2394,7 @@
         <v>22</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="C12" t="s">
         <v>41</v>
@@ -2403,55 +2403,52 @@
         <v>66</v>
       </c>
       <c r="E12">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="F12">
-        <v>2396</v>
+        <v>1313</v>
       </c>
       <c r="G12" t="s">
-        <v>78</v>
+        <v>72</v>
+      </c>
+      <c r="H12">
+        <v>750000</v>
       </c>
       <c r="I12" t="s">
-        <v>85</v>
+        <v>81</v>
       </c>
       <c r="J12">
-        <v>89</v>
+        <v>88.90000000000001</v>
       </c>
       <c r="K12">
-        <v>80</v>
+        <v>27</v>
       </c>
       <c r="L12">
-        <v>63</v>
+        <v>19</v>
       </c>
       <c r="M12">
-        <v>17</v>
+        <v>5</v>
       </c>
       <c r="N12">
-        <v>47.1</v>
+        <v>20</v>
       </c>
       <c r="O12">
-        <v>0.13</v>
+        <v>0.08</v>
       </c>
       <c r="P12">
-        <v>20</v>
-      </c>
-      <c r="Q12">
-        <v>96.59999999999999</v>
-      </c>
-      <c r="R12">
-        <v>102</v>
+        <v>44.4</v>
       </c>
       <c r="S12">
         <v>0</v>
       </c>
       <c r="T12">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="U12">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V12">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="13" spans="1:22">
@@ -2459,7 +2456,7 @@
         <v>22</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>23</v>
       </c>
       <c r="C13" t="s">
         <v>42</v>
@@ -2468,49 +2465,46 @@
         <v>67</v>
       </c>
       <c r="E13">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="F13">
-        <v>1313</v>
+        <v>1761</v>
       </c>
       <c r="G13" t="s">
-        <v>73</v>
-      </c>
-      <c r="H13">
-        <v>750000</v>
+        <v>78</v>
       </c>
       <c r="I13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J13">
-        <v>88.90000000000001</v>
+        <v>88</v>
       </c>
       <c r="K13">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="L13">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="M13">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="N13">
-        <v>20</v>
+        <v>16.7</v>
       </c>
       <c r="O13">
-        <v>0.08</v>
+        <v>0.16</v>
       </c>
       <c r="P13">
-        <v>44.4</v>
+        <v>30.2</v>
       </c>
       <c r="S13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="U13">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="V13">
         <v>0</v>
@@ -2521,52 +2515,61 @@
         <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="C14" t="s">
         <v>43</v>
       </c>
       <c r="D14" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="E14">
-        <v>20</v>
+        <v>32</v>
       </c>
       <c r="F14">
-        <v>1761</v>
+        <v>1569</v>
       </c>
       <c r="G14" t="s">
-        <v>79</v>
+        <v>72</v>
+      </c>
+      <c r="H14">
+        <v>500000</v>
       </c>
       <c r="I14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J14">
-        <v>88</v>
+        <v>87.59999999999999</v>
       </c>
       <c r="K14">
-        <v>42</v>
+        <v>21</v>
       </c>
       <c r="L14">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="M14">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="N14">
-        <v>16.7</v>
+        <v>33.3</v>
       </c>
       <c r="O14">
-        <v>0.16</v>
+        <v>0.11</v>
       </c>
       <c r="P14">
-        <v>30.2</v>
+        <v>46.4</v>
+      </c>
+      <c r="Q14">
+        <v>79.2</v>
+      </c>
+      <c r="R14">
+        <v>18</v>
       </c>
       <c r="S14">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="T14">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="U14">
         <v>3</v>
@@ -2580,64 +2583,61 @@
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
         <v>44</v>
       </c>
       <c r="D15" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E15">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="F15">
-        <v>1569</v>
+        <v>2186</v>
       </c>
       <c r="G15" t="s">
-        <v>73</v>
-      </c>
-      <c r="H15">
-        <v>500000</v>
+        <v>72</v>
       </c>
       <c r="I15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J15">
-        <v>87.59999999999999</v>
+        <v>86.7</v>
       </c>
       <c r="K15">
-        <v>21</v>
+        <v>42</v>
       </c>
       <c r="L15">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="M15">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="N15">
-        <v>33.3</v>
+        <v>20</v>
       </c>
       <c r="O15">
         <v>0.11</v>
       </c>
       <c r="P15">
-        <v>46.4</v>
+        <v>32.3</v>
       </c>
       <c r="Q15">
-        <v>79.2</v>
+        <v>92.90000000000001</v>
       </c>
       <c r="R15">
-        <v>18</v>
+        <v>66</v>
       </c>
       <c r="S15">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="T15">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="U15">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="V15">
         <v>0</v>
@@ -2648,64 +2648,67 @@
         <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>24</v>
+        <v>30</v>
       </c>
       <c r="C16" t="s">
         <v>45</v>
       </c>
       <c r="D16" t="s">
-        <v>69</v>
+        <v>57</v>
       </c>
       <c r="E16">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="F16">
-        <v>2186</v>
+        <v>2301</v>
       </c>
       <c r="G16" t="s">
         <v>73</v>
       </c>
+      <c r="H16">
+        <v>125000</v>
+      </c>
       <c r="I16" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="J16">
-        <v>86.7</v>
+        <v>84.5</v>
       </c>
       <c r="K16">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="L16">
-        <v>30</v>
+        <v>17</v>
       </c>
       <c r="M16">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N16">
-        <v>20</v>
+        <v>100</v>
       </c>
       <c r="O16">
-        <v>0.11</v>
+        <v>0.12</v>
       </c>
       <c r="P16">
-        <v>32.3</v>
+        <v>32</v>
       </c>
       <c r="Q16">
-        <v>92.90000000000001</v>
+        <v>61</v>
       </c>
       <c r="R16">
-        <v>66</v>
+        <v>6</v>
       </c>
       <c r="S16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="T16">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U16">
         <v>2</v>
       </c>
       <c r="V16">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="17" spans="1:22">
@@ -2719,61 +2722,55 @@
         <v>46</v>
       </c>
       <c r="D17" t="s">
-        <v>57</v>
+        <v>69</v>
       </c>
       <c r="E17">
         <v>29</v>
       </c>
       <c r="F17">
-        <v>2301</v>
+        <v>1941</v>
       </c>
       <c r="G17" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H17">
-        <v>125000</v>
+        <v>900000</v>
       </c>
       <c r="I17" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="J17">
-        <v>84.5</v>
+        <v>84.2</v>
       </c>
       <c r="K17">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="L17">
         <v>17</v>
       </c>
       <c r="M17">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="N17">
-        <v>100</v>
+        <v>66.7</v>
       </c>
       <c r="O17">
-        <v>0.12</v>
+        <v>0.08</v>
       </c>
       <c r="P17">
-        <v>32</v>
-      </c>
-      <c r="Q17">
-        <v>61</v>
-      </c>
-      <c r="R17">
-        <v>6</v>
+        <v>48.3</v>
       </c>
       <c r="S17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="T17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U17">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="V17">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="18" spans="1:22">
@@ -2781,7 +2778,7 @@
         <v>22</v>
       </c>
       <c r="B18" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C18" t="s">
         <v>47</v>
@@ -2793,49 +2790,49 @@
         <v>29</v>
       </c>
       <c r="F18">
-        <v>1941</v>
+        <v>1435</v>
       </c>
       <c r="G18" t="s">
         <v>73</v>
       </c>
       <c r="H18">
-        <v>900000</v>
+        <v>1000000</v>
       </c>
       <c r="I18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J18">
         <v>84.2</v>
       </c>
       <c r="K18">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="L18">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="M18">
+        <v>9</v>
+      </c>
+      <c r="N18">
+        <v>11.1</v>
+      </c>
+      <c r="O18">
+        <v>0.07000000000000001</v>
+      </c>
+      <c r="P18">
+        <v>36.4</v>
+      </c>
+      <c r="S18">
+        <v>0</v>
+      </c>
+      <c r="T18">
         <v>3</v>
       </c>
-      <c r="N18">
-        <v>66.7</v>
-      </c>
-      <c r="O18">
-        <v>0.08</v>
-      </c>
-      <c r="P18">
-        <v>48.3</v>
-      </c>
-      <c r="S18">
-        <v>0</v>
-      </c>
-      <c r="T18">
-        <v>0</v>
-      </c>
       <c r="U18">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V18">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19" spans="1:22">
@@ -2843,61 +2840,67 @@
         <v>22</v>
       </c>
       <c r="B19" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C19" t="s">
         <v>48</v>
       </c>
       <c r="D19" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E19">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="F19">
-        <v>1435</v>
+        <v>1015</v>
       </c>
       <c r="G19" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H19">
-        <v>1000000</v>
+        <v>200000</v>
       </c>
       <c r="I19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J19">
-        <v>84.2</v>
+        <v>83.90000000000001</v>
       </c>
       <c r="K19">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="L19">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="M19">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="N19">
-        <v>11.1</v>
+        <v>50</v>
       </c>
       <c r="O19">
-        <v>0.07000000000000001</v>
+        <v>0.11</v>
       </c>
       <c r="P19">
-        <v>36.4</v>
+        <v>21</v>
+      </c>
+      <c r="Q19">
+        <v>94.40000000000001</v>
+      </c>
+      <c r="R19">
+        <v>97</v>
       </c>
       <c r="S19">
         <v>0</v>
       </c>
       <c r="T19">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="U19">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V19">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="20" spans="1:22">
@@ -2905,67 +2908,61 @@
         <v>22</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C20" t="s">
         <v>49</v>
       </c>
       <c r="D20" t="s">
-        <v>71</v>
+        <v>65</v>
       </c>
       <c r="E20">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="F20">
-        <v>1015</v>
+        <v>1877</v>
       </c>
       <c r="G20" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="H20">
-        <v>200000</v>
+        <v>400000</v>
       </c>
       <c r="I20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J20">
-        <v>83.90000000000001</v>
+        <v>83.09999999999999</v>
       </c>
       <c r="K20">
-        <v>19</v>
+        <v>29</v>
       </c>
       <c r="L20">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="M20">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="N20">
-        <v>50</v>
+        <v>0</v>
       </c>
       <c r="O20">
-        <v>0.11</v>
+        <v>0.14</v>
       </c>
       <c r="P20">
-        <v>21</v>
-      </c>
-      <c r="Q20">
-        <v>94.40000000000001</v>
-      </c>
-      <c r="R20">
-        <v>97</v>
+        <v>40</v>
       </c>
       <c r="S20">
         <v>0</v>
       </c>
       <c r="T20">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="U20">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V20">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="21" spans="1:22">
@@ -2973,13 +2970,13 @@
         <v>22</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C21" t="s">
         <v>50</v>
       </c>
       <c r="D21" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E21">
         <v>31</v>
@@ -2988,13 +2985,13 @@
         <v>1972</v>
       </c>
       <c r="G21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H21">
         <v>250000</v>
       </c>
       <c r="I21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J21">
         <v>83.09999999999999</v>
@@ -3035,58 +3032,61 @@
         <v>22</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="C22" t="s">
         <v>51</v>
       </c>
       <c r="D22" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="E22">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F22">
-        <v>1877</v>
+        <v>2285</v>
       </c>
       <c r="G22" t="s">
-        <v>75</v>
-      </c>
-      <c r="H22">
-        <v>400000</v>
+        <v>73</v>
       </c>
       <c r="I22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J22">
-        <v>83.09999999999999</v>
+        <v>81.8</v>
       </c>
       <c r="K22">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="L22">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="M22">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="N22">
         <v>0</v>
       </c>
       <c r="O22">
-        <v>0.14</v>
+        <v>0.21</v>
       </c>
       <c r="P22">
-        <v>40</v>
+        <v>38.8</v>
+      </c>
+      <c r="Q22">
+        <v>65.3</v>
+      </c>
+      <c r="R22">
+        <v>17</v>
       </c>
       <c r="S22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="T22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="U22">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="V22">
         <v>0</v>
@@ -3103,28 +3103,31 @@
         <v>52</v>
       </c>
       <c r="D23" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
       <c r="E23">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="F23">
-        <v>2285</v>
+        <v>1133</v>
       </c>
       <c r="G23" t="s">
-        <v>74</v>
+        <v>73</v>
+      </c>
+      <c r="H23">
+        <v>1000000</v>
       </c>
       <c r="I23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J23">
-        <v>81.8</v>
+        <v>81.09999999999999</v>
       </c>
       <c r="K23">
-        <v>42</v>
+        <v>20</v>
       </c>
       <c r="L23">
-        <v>14</v>
+        <v>10</v>
       </c>
       <c r="M23">
         <v>2</v>
@@ -3133,25 +3136,25 @@
         <v>0</v>
       </c>
       <c r="O23">
-        <v>0.21</v>
+        <v>0.12</v>
       </c>
       <c r="P23">
-        <v>38.8</v>
+        <v>35</v>
       </c>
       <c r="Q23">
-        <v>65.3</v>
+        <v>81.2</v>
       </c>
       <c r="R23">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="S23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="T23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="U23">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="V23">
         <v>0</v>
@@ -3162,55 +3165,49 @@
         <v>22</v>
       </c>
       <c r="B24" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C24" t="s">
         <v>53</v>
       </c>
       <c r="D24" t="s">
-        <v>64</v>
+        <v>71</v>
       </c>
       <c r="E24">
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="F24">
-        <v>1133</v>
+        <v>2014</v>
       </c>
       <c r="G24" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="H24">
-        <v>1000000</v>
+        <v>750000</v>
       </c>
       <c r="I24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J24">
-        <v>81.09999999999999</v>
+        <v>79.90000000000001</v>
       </c>
       <c r="K24">
-        <v>20</v>
+        <v>35</v>
       </c>
       <c r="L24">
-        <v>10</v>
+        <v>27</v>
       </c>
       <c r="M24">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="N24">
         <v>0</v>
       </c>
       <c r="O24">
-        <v>0.12</v>
+        <v>0.09</v>
       </c>
       <c r="P24">
-        <v>35</v>
-      </c>
-      <c r="Q24">
-        <v>81.2</v>
-      </c>
-      <c r="R24">
-        <v>21</v>
+        <v>29.8</v>
       </c>
       <c r="S24">
         <v>1</v>
@@ -3230,58 +3227,58 @@
         <v>22</v>
       </c>
       <c r="B25" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="C25" t="s">
         <v>54</v>
       </c>
       <c r="D25" t="s">
-        <v>72</v>
+        <v>58</v>
       </c>
       <c r="E25">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="F25">
-        <v>2014</v>
+        <v>2238</v>
       </c>
       <c r="G25" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="H25">
-        <v>750000</v>
+        <v>100000</v>
       </c>
       <c r="I25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J25">
-        <v>79.90000000000001</v>
+        <v>79.5</v>
       </c>
       <c r="K25">
-        <v>35</v>
+        <v>28</v>
       </c>
       <c r="L25">
-        <v>27</v>
+        <v>7</v>
       </c>
       <c r="M25">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="N25">
-        <v>0</v>
+        <v>100</v>
       </c>
       <c r="O25">
-        <v>0.09</v>
+        <v>0.08</v>
       </c>
       <c r="P25">
-        <v>29.8</v>
+        <v>34.4</v>
       </c>
       <c r="S25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="U25">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="V25">
         <v>0</v>
@@ -3292,61 +3289,55 @@
         <v>22</v>
       </c>
       <c r="B26" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C26" t="s">
         <v>55</v>
       </c>
       <c r="D26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="E26">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="F26">
-        <v>2238</v>
-      </c>
-      <c r="G26" t="s">
-        <v>80</v>
-      </c>
-      <c r="H26">
-        <v>100000</v>
+        <v>903</v>
       </c>
       <c r="I26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J26">
-        <v>79.5</v>
+        <v>78.40000000000001</v>
       </c>
       <c r="K26">
-        <v>28</v>
+        <v>4</v>
       </c>
       <c r="L26">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="M26">
+        <v>3</v>
+      </c>
+      <c r="N26">
+        <v>66.7</v>
+      </c>
+      <c r="O26">
+        <v>0.03</v>
+      </c>
+      <c r="P26">
+        <v>37.5</v>
+      </c>
+      <c r="S26">
         <v>1</v>
       </c>
-      <c r="N26">
-        <v>100</v>
-      </c>
-      <c r="O26">
-        <v>0.08</v>
-      </c>
-      <c r="P26">
-        <v>34.4</v>
-      </c>
-      <c r="S26">
-        <v>0</v>
-      </c>
       <c r="T26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="U26">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="V26">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3388,40 +3379,40 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>91</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="P1" s="1" t="s">
         <v>92</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>93</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="R1" s="1" t="s">
         <v>94</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="T1" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="U1" s="1" t="s">
         <v>97</v>
-      </c>
-      <c r="U1" s="1" t="s">
-        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:21">
@@ -3429,13 +3420,13 @@
         <v>22</v>
       </c>
       <c r="B2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E2">
         <v>33</v>
@@ -3444,13 +3435,13 @@
         <v>1988</v>
       </c>
       <c r="G2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H2">
         <v>900000</v>
       </c>
       <c r="I2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J2">
         <v>92.5</v>
@@ -3488,10 +3479,10 @@
         <v>22</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="D3" t="s">
         <v>57</v>
@@ -3503,10 +3494,10 @@
         <v>2612</v>
       </c>
       <c r="G3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J3">
         <v>90.7</v>
@@ -3553,10 +3544,10 @@
         <v>29</v>
       </c>
       <c r="C4" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="D4" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E4">
         <v>31</v>
@@ -3565,13 +3556,13 @@
         <v>1585</v>
       </c>
       <c r="G4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H4">
         <v>400000</v>
       </c>
       <c r="I4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J4">
         <v>88.3</v>
@@ -3618,10 +3609,10 @@
         <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="D5" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E5">
         <v>28</v>
@@ -3630,13 +3621,13 @@
         <v>1299</v>
       </c>
       <c r="G5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H5">
         <v>800000</v>
       </c>
       <c r="I5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J5">
         <v>88</v>
@@ -3674,10 +3665,10 @@
         <v>22</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="D6" t="s">
         <v>59</v>
@@ -3692,7 +3683,7 @@
         <v>128</v>
       </c>
       <c r="I6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J6">
         <v>85</v>
@@ -3733,10 +3724,10 @@
         <v>25</v>
       </c>
       <c r="C7" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="D7" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E7">
         <v>24</v>
@@ -3748,7 +3739,7 @@
         <v>129</v>
       </c>
       <c r="I7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J7">
         <v>84.09999999999999</v>
@@ -3786,13 +3777,13 @@
         <v>22</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C8" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="D8" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E8">
         <v>31</v>
@@ -3801,13 +3792,13 @@
         <v>1645</v>
       </c>
       <c r="G8" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H8">
         <v>600000</v>
       </c>
       <c r="I8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J8">
         <v>84.09999999999999</v>
@@ -3851,13 +3842,13 @@
         <v>22</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C9" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E9">
         <v>29</v>
@@ -3866,10 +3857,10 @@
         <v>1236</v>
       </c>
       <c r="G9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J9">
         <v>83.09999999999999</v>
@@ -3913,10 +3904,10 @@
         <v>26</v>
       </c>
       <c r="C10" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="D10" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E10">
         <v>24</v>
@@ -3928,7 +3919,7 @@
         <v>130</v>
       </c>
       <c r="I10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J10">
         <v>82.09999999999999</v>
@@ -3966,10 +3957,10 @@
         <v>29</v>
       </c>
       <c r="C11" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="D11" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E11">
         <v>27</v>
@@ -3978,13 +3969,13 @@
         <v>2236</v>
       </c>
       <c r="G11" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="H11">
         <v>300000</v>
       </c>
       <c r="I11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J11">
         <v>80.8</v>
@@ -4031,10 +4022,10 @@
         <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D12" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E12">
         <v>22</v>
@@ -4043,10 +4034,10 @@
         <v>1515</v>
       </c>
       <c r="G12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J12">
         <v>80.40000000000001</v>
@@ -4087,7 +4078,7 @@
         <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D13" t="s">
         <v>57</v>
@@ -4099,13 +4090,13 @@
         <v>2420</v>
       </c>
       <c r="G13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H13">
         <v>400000</v>
       </c>
       <c r="I13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J13">
         <v>79.90000000000001</v>
@@ -4143,13 +4134,13 @@
         <v>22</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>126</v>
       </c>
       <c r="E14">
         <v>30</v>
@@ -4158,10 +4149,10 @@
         <v>1009</v>
       </c>
       <c r="G14" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J14">
         <v>79.8</v>
@@ -4199,13 +4190,13 @@
         <v>22</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C15" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D15" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E15">
         <v>30</v>
@@ -4214,10 +4205,10 @@
         <v>1733</v>
       </c>
       <c r="G15" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J15">
         <v>77.7</v>
@@ -4261,13 +4252,13 @@
         <v>22</v>
       </c>
       <c r="B16" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C16" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E16">
         <v>22</v>
@@ -4276,10 +4267,10 @@
         <v>1877</v>
       </c>
       <c r="G16" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J16">
         <v>77.40000000000001</v>
@@ -4326,10 +4317,10 @@
         <v>29</v>
       </c>
       <c r="C17" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E17">
         <v>27</v>
@@ -4338,7 +4329,7 @@
         <v>1800</v>
       </c>
       <c r="G17" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="I17" t="s">
         <v>131</v>
@@ -4382,7 +4373,7 @@
         <v>25</v>
       </c>
       <c r="C18" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D18" t="s">
         <v>59</v>
@@ -4394,10 +4385,10 @@
         <v>1438</v>
       </c>
       <c r="G18" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J18">
         <v>74.8</v>
@@ -4444,7 +4435,7 @@
         <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D19" t="s">
         <v>127</v>
@@ -4456,13 +4447,13 @@
         <v>908</v>
       </c>
       <c r="G19" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H19">
         <v>250000</v>
       </c>
       <c r="I19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J19">
         <v>72.90000000000001</v>
@@ -4503,10 +4494,10 @@
         <v>29</v>
       </c>
       <c r="C20" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D20" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E20">
         <v>28</v>
@@ -4515,13 +4506,13 @@
         <v>2493</v>
       </c>
       <c r="G20" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H20">
         <v>1200000</v>
       </c>
       <c r="I20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J20">
         <v>72.90000000000001</v>
@@ -4562,7 +4553,7 @@
         <v>30</v>
       </c>
       <c r="C21" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="D21" t="s">
         <v>57</v>
@@ -4574,13 +4565,13 @@
         <v>2301</v>
       </c>
       <c r="G21" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H21">
         <v>125000</v>
       </c>
       <c r="I21" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="J21">
         <v>72.09999999999999</v>
@@ -4627,10 +4618,10 @@
         <v>23</v>
       </c>
       <c r="C22" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D22" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E22">
         <v>28</v>
@@ -4639,13 +4630,13 @@
         <v>960</v>
       </c>
       <c r="G22" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="H22">
         <v>500000</v>
       </c>
       <c r="I22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J22">
         <v>71.5</v>
@@ -4692,10 +4683,10 @@
         <v>29</v>
       </c>
       <c r="C23" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D23" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E23">
         <v>27</v>
@@ -4704,10 +4695,10 @@
         <v>1728</v>
       </c>
       <c r="G23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="I23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J23">
         <v>69.90000000000001</v>
@@ -4754,10 +4745,10 @@
         <v>29</v>
       </c>
       <c r="C24" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D24" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E24">
         <v>33</v>
@@ -4766,7 +4757,7 @@
         <v>1408</v>
       </c>
       <c r="G24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H24">
         <v>2000000</v>
@@ -4813,10 +4804,10 @@
         <v>29</v>
       </c>
       <c r="C25" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D25" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E25">
         <v>20</v>
@@ -4825,10 +4816,10 @@
         <v>1285</v>
       </c>
       <c r="G25" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="I25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J25">
         <v>67.7</v>
@@ -4863,10 +4854,10 @@
         <v>22</v>
       </c>
       <c r="B26" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C26" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D26" t="s">
         <v>56</v>
@@ -4878,13 +4869,13 @@
         <v>1710</v>
       </c>
       <c r="G26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H26">
         <v>450000</v>
       </c>
       <c r="I26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J26">
         <v>67.3</v>
@@ -4988,7 +4979,7 @@
         <v>133</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
         <v>134</v>
@@ -5003,7 +4994,7 @@
         <v>1682</v>
       </c>
       <c r="G2" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -5053,7 +5044,7 @@
         <v>1920</v>
       </c>
       <c r="G3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H3">
         <v>0</v>
@@ -5088,7 +5079,7 @@
         <v>133</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
         <v>136</v>
@@ -5103,7 +5094,7 @@
         <v>1061</v>
       </c>
       <c r="G4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -5138,7 +5129,7 @@
         <v>133</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
         <v>137</v>
@@ -5153,7 +5144,7 @@
         <v>1914</v>
       </c>
       <c r="G5" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H5">
         <v>0</v>
@@ -5203,13 +5194,13 @@
         <v>980</v>
       </c>
       <c r="G6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J6">
         <v>92.3</v>
@@ -5259,7 +5250,7 @@
         <v>0</v>
       </c>
       <c r="I7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J7">
         <v>88.8</v>
@@ -5288,7 +5279,7 @@
         <v>133</v>
       </c>
       <c r="B8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
         <v>140</v>
@@ -5353,13 +5344,13 @@
         <v>933</v>
       </c>
       <c r="G9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J9">
         <v>85.2</v>
@@ -5459,7 +5450,7 @@
         <v>1500000</v>
       </c>
       <c r="I11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J11">
         <v>83.7</v>
@@ -5503,13 +5494,13 @@
         <v>1691</v>
       </c>
       <c r="G12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H12">
         <v>1200000</v>
       </c>
       <c r="I12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J12">
         <v>81</v>
@@ -5553,7 +5544,7 @@
         <v>1005</v>
       </c>
       <c r="G13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H13">
         <v>1000000</v>
@@ -5588,7 +5579,7 @@
         <v>133</v>
       </c>
       <c r="B14" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C14" t="s">
         <v>146</v>
@@ -5653,13 +5644,13 @@
         <v>907</v>
       </c>
       <c r="G15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H15">
         <v>450000</v>
       </c>
       <c r="I15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J15">
         <v>80.40000000000001</v>
@@ -5809,7 +5800,7 @@
         <v>0</v>
       </c>
       <c r="I18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J18">
         <v>77.2</v>
@@ -5903,13 +5894,13 @@
         <v>1582</v>
       </c>
       <c r="G20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H20">
         <v>300000</v>
       </c>
       <c r="I20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J20">
         <v>76</v>
@@ -5959,7 +5950,7 @@
         <v>0</v>
       </c>
       <c r="I21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J21">
         <v>73.8</v>
@@ -6003,13 +5994,13 @@
         <v>1579</v>
       </c>
       <c r="G22" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H22">
         <v>0</v>
       </c>
       <c r="I22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J22">
         <v>72.8</v>
@@ -6059,7 +6050,7 @@
         <v>0</v>
       </c>
       <c r="I23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J23">
         <v>71.7</v>
@@ -6103,7 +6094,7 @@
         <v>1913</v>
       </c>
       <c r="G24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H24">
         <v>2000000</v>
@@ -6159,7 +6150,7 @@
         <v>0</v>
       </c>
       <c r="I25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J25">
         <v>71.2</v>
@@ -6203,13 +6194,13 @@
         <v>1438</v>
       </c>
       <c r="G26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H26">
         <v>900000</v>
       </c>
       <c r="I26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J26">
         <v>70.90000000000001</v>
@@ -6272,22 +6263,22 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -6295,7 +6286,7 @@
         <v>133</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s">
         <v>187</v>
@@ -6310,13 +6301,13 @@
         <v>1633</v>
       </c>
       <c r="G2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H2">
         <v>1000000</v>
       </c>
       <c r="I2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J2">
         <v>96.8</v>
@@ -6342,7 +6333,7 @@
         <v>133</v>
       </c>
       <c r="B3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C3" t="s">
         <v>188</v>
@@ -6357,13 +6348,13 @@
         <v>2261</v>
       </c>
       <c r="G3" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H3">
         <v>250000</v>
       </c>
       <c r="I3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J3">
         <v>93.59999999999999</v>
@@ -6389,7 +6380,7 @@
         <v>133</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
         <v>189</v>
@@ -6410,7 +6401,7 @@
         <v>1500000</v>
       </c>
       <c r="I4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J4">
         <v>93.59999999999999</v>
@@ -6436,7 +6427,7 @@
         <v>133</v>
       </c>
       <c r="B5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" t="s">
         <v>190</v>
@@ -6451,13 +6442,13 @@
         <v>1549</v>
       </c>
       <c r="G5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H5">
         <v>400000</v>
       </c>
       <c r="I5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J5">
         <v>90.5</v>
@@ -6498,13 +6489,13 @@
         <v>1435</v>
       </c>
       <c r="G6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H6">
         <v>0</v>
       </c>
       <c r="I6" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J6">
         <v>85.59999999999999</v>
@@ -6530,7 +6521,7 @@
         <v>133</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C7" t="s">
         <v>192</v>
@@ -6545,13 +6536,13 @@
         <v>1694</v>
       </c>
       <c r="G7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H7">
         <v>100000</v>
       </c>
       <c r="I7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J7">
         <v>85.59999999999999</v>
@@ -6577,7 +6568,7 @@
         <v>133</v>
       </c>
       <c r="B8" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C8" t="s">
         <v>193</v>
@@ -6592,13 +6583,13 @@
         <v>1711</v>
       </c>
       <c r="G8" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H8">
         <v>100000</v>
       </c>
       <c r="I8" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J8">
         <v>85.5</v>
@@ -6624,7 +6615,7 @@
         <v>133</v>
       </c>
       <c r="B9" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C9" t="s">
         <v>194</v>
@@ -6639,7 +6630,7 @@
         <v>1708</v>
       </c>
       <c r="G9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H9">
         <v>850000</v>
@@ -6671,7 +6662,7 @@
         <v>133</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C10" t="s">
         <v>195</v>
@@ -6686,13 +6677,13 @@
         <v>1618</v>
       </c>
       <c r="G10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H10">
         <v>0</v>
       </c>
       <c r="I10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J10">
         <v>83.7</v>
@@ -6718,7 +6709,7 @@
         <v>133</v>
       </c>
       <c r="B11" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C11" t="s">
         <v>196</v>
@@ -6739,7 +6730,7 @@
         <v>0</v>
       </c>
       <c r="I11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J11">
         <v>82.3</v>
@@ -6812,7 +6803,7 @@
         <v>133</v>
       </c>
       <c r="B13" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C13" t="s">
         <v>198</v>
@@ -6833,7 +6824,7 @@
         <v>2000000</v>
       </c>
       <c r="I13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J13">
         <v>78.90000000000001</v>
@@ -6859,7 +6850,7 @@
         <v>133</v>
       </c>
       <c r="B14" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C14" t="s">
         <v>199</v>
@@ -6874,13 +6865,13 @@
         <v>1931</v>
       </c>
       <c r="G14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H14">
         <v>250000</v>
       </c>
       <c r="I14" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J14">
         <v>78.7</v>
@@ -6927,7 +6918,7 @@
         <v>0</v>
       </c>
       <c r="I15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J15">
         <v>77.3</v>
@@ -7068,7 +7059,7 @@
         <v>0</v>
       </c>
       <c r="I18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J18">
         <v>67</v>
@@ -7094,7 +7085,7 @@
         <v>133</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C19" t="s">
         <v>203</v>
@@ -7115,7 +7106,7 @@
         <v>0</v>
       </c>
       <c r="I19" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J19">
         <v>65.2</v>
@@ -7156,13 +7147,13 @@
         <v>1868</v>
       </c>
       <c r="G20" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H20">
         <v>1500000</v>
       </c>
       <c r="I20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J20">
         <v>64.7</v>
@@ -7188,7 +7179,7 @@
         <v>133</v>
       </c>
       <c r="B21" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C21" t="s">
         <v>205</v>
@@ -7203,13 +7194,13 @@
         <v>1962</v>
       </c>
       <c r="G21" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H21">
         <v>1000000</v>
       </c>
       <c r="I21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J21">
         <v>64.2</v>
@@ -7256,7 +7247,7 @@
         <v>0</v>
       </c>
       <c r="I22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J22">
         <v>64.09999999999999</v>
@@ -7282,7 +7273,7 @@
         <v>133</v>
       </c>
       <c r="B23" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C23" t="s">
         <v>207</v>
@@ -7300,7 +7291,7 @@
         <v>0</v>
       </c>
       <c r="I23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J23">
         <v>63.8</v>
@@ -7326,7 +7317,7 @@
         <v>133</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C24" t="s">
         <v>208</v>
@@ -7341,13 +7332,13 @@
         <v>1620</v>
       </c>
       <c r="G24" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H24">
         <v>1000000</v>
       </c>
       <c r="I24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J24">
         <v>62.5</v>
@@ -7373,7 +7364,7 @@
         <v>133</v>
       </c>
       <c r="B25" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C25" t="s">
         <v>209</v>
@@ -7388,13 +7379,13 @@
         <v>1452</v>
       </c>
       <c r="G25" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H25">
         <v>1000000</v>
       </c>
       <c r="I25" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J25">
         <v>62</v>
@@ -7420,7 +7411,7 @@
         <v>133</v>
       </c>
       <c r="B26" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C26" t="s">
         <v>210</v>
@@ -7435,13 +7426,13 @@
         <v>1476</v>
       </c>
       <c r="G26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H26">
         <v>1300000</v>
       </c>
       <c r="I26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J26">
         <v>61.4</v>
@@ -7542,7 +7533,7 @@
         <v>1422</v>
       </c>
       <c r="G2" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H2">
         <v>0</v>
@@ -7595,7 +7586,7 @@
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J3">
         <v>96</v>
@@ -7621,7 +7612,7 @@
     </row>
     <row r="4" spans="1:16">
       <c r="A4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B4" t="s">
         <v>24</v>
@@ -7639,13 +7630,13 @@
         <v>939</v>
       </c>
       <c r="G4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H4">
         <v>175000</v>
       </c>
       <c r="I4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J4">
         <v>96</v>
@@ -7689,13 +7680,13 @@
         <v>1589</v>
       </c>
       <c r="G5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H5">
         <v>0</v>
       </c>
       <c r="I5" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J5">
         <v>95.59999999999999</v>
@@ -7721,7 +7712,7 @@
     </row>
     <row r="6" spans="1:16">
       <c r="A6" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B6" t="s">
         <v>26</v>
@@ -7739,7 +7730,7 @@
         <v>1085</v>
       </c>
       <c r="G6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H6">
         <v>200000</v>
@@ -7774,7 +7765,7 @@
         <v>219</v>
       </c>
       <c r="B7" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C7" t="s">
         <v>231</v>
@@ -7789,7 +7780,7 @@
         <v>1128</v>
       </c>
       <c r="G7" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H7">
         <v>800000</v>
@@ -7824,7 +7815,7 @@
         <v>220</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C8" t="s">
         <v>232</v>
@@ -7936,7 +7927,7 @@
         <v>2055</v>
       </c>
       <c r="G10" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -7971,7 +7962,7 @@
         <v>221</v>
       </c>
       <c r="B11" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" t="s">
         <v>235</v>
@@ -8036,7 +8027,7 @@
         <v>1602</v>
       </c>
       <c r="G12" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -8086,7 +8077,7 @@
         <v>1809</v>
       </c>
       <c r="G13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H13">
         <v>0</v>
@@ -8136,7 +8127,7 @@
         <v>2172</v>
       </c>
       <c r="G14" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -8171,7 +8162,7 @@
         <v>219</v>
       </c>
       <c r="B15" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C15" t="s">
         <v>239</v>
@@ -8186,7 +8177,7 @@
         <v>1726</v>
       </c>
       <c r="G15" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H15">
         <v>450000</v>
@@ -8236,13 +8227,13 @@
         <v>2156</v>
       </c>
       <c r="G16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H16">
         <v>0</v>
       </c>
       <c r="I16" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J16">
         <v>94.09999999999999</v>
@@ -8289,7 +8280,7 @@
         <v>0</v>
       </c>
       <c r="I17" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J17">
         <v>94.09999999999999</v>
@@ -8333,7 +8324,7 @@
         <v>1629</v>
       </c>
       <c r="G18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H18">
         <v>0</v>
@@ -8415,7 +8406,7 @@
         <v>220</v>
       </c>
       <c r="B20" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C20" t="s">
         <v>244</v>
@@ -8477,7 +8468,7 @@
         <v>1403</v>
       </c>
       <c r="G21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H21">
         <v>500000</v>
@@ -8530,7 +8521,7 @@
         <v>1500000</v>
       </c>
       <c r="I22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J22">
         <v>93.40000000000001</v>
@@ -8624,13 +8615,13 @@
         <v>1768</v>
       </c>
       <c r="G24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H24">
         <v>700000</v>
       </c>
       <c r="I24" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J24">
         <v>93.40000000000001</v>
@@ -8721,7 +8712,7 @@
         <v>1049</v>
       </c>
       <c r="G26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H26">
         <v>0</v>
@@ -8790,30 +8781,30 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:15">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C2" t="s">
         <v>278</v>
@@ -8828,7 +8819,7 @@
         <v>1528</v>
       </c>
       <c r="G2" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H2">
         <v>500000</v>
@@ -8860,7 +8851,7 @@
         <v>221</v>
       </c>
       <c r="B3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C3" t="s">
         <v>279</v>
@@ -8904,7 +8895,7 @@
         <v>220</v>
       </c>
       <c r="B4" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C4" t="s">
         <v>280</v>
@@ -8919,13 +8910,13 @@
         <v>2177</v>
       </c>
       <c r="G4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H4">
         <v>0</v>
       </c>
       <c r="I4" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="J4">
         <v>94.40000000000001</v>
@@ -8951,7 +8942,7 @@
         <v>222</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C5" t="s">
         <v>281</v>
@@ -8966,7 +8957,7 @@
         <v>2099</v>
       </c>
       <c r="G5" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H5">
         <v>75000</v>
@@ -8998,7 +8989,7 @@
         <v>218</v>
       </c>
       <c r="B6" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C6" t="s">
         <v>282</v>
@@ -9013,7 +9004,7 @@
         <v>1911</v>
       </c>
       <c r="G6" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H6">
         <v>0</v>
@@ -9045,7 +9036,7 @@
         <v>222</v>
       </c>
       <c r="B7" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C7" t="s">
         <v>283</v>
@@ -9060,7 +9051,7 @@
         <v>2131</v>
       </c>
       <c r="G7" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H7">
         <v>175000</v>
@@ -9107,13 +9098,13 @@
         <v>1133</v>
       </c>
       <c r="G8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H8">
         <v>0</v>
       </c>
       <c r="I8" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J8">
         <v>92.09999999999999</v>
@@ -9154,7 +9145,7 @@
         <v>2232</v>
       </c>
       <c r="G9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H9">
         <v>0</v>
@@ -9186,7 +9177,7 @@
         <v>221</v>
       </c>
       <c r="B10" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C10" t="s">
         <v>286</v>
@@ -9201,7 +9192,7 @@
         <v>1975</v>
       </c>
       <c r="G10" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H10">
         <v>10000</v>
@@ -9233,7 +9224,7 @@
         <v>219</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C11" t="s">
         <v>287</v>
@@ -9292,7 +9283,7 @@
         <v>1782</v>
       </c>
       <c r="G12" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H12">
         <v>0</v>
@@ -9324,7 +9315,7 @@
         <v>217</v>
       </c>
       <c r="B13" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C13" t="s">
         <v>289</v>
@@ -9339,13 +9330,13 @@
         <v>2059</v>
       </c>
       <c r="G13" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H13">
         <v>0</v>
       </c>
       <c r="I13" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J13">
         <v>90.90000000000001</v>
@@ -9371,7 +9362,7 @@
         <v>222</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
         <v>290</v>
@@ -9415,7 +9406,7 @@
         <v>224</v>
       </c>
       <c r="B15" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C15" t="s">
         <v>291</v>
@@ -9459,7 +9450,7 @@
         <v>216</v>
       </c>
       <c r="B16" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C16" t="s">
         <v>292</v>
@@ -9474,7 +9465,7 @@
         <v>1287</v>
       </c>
       <c r="G16" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H16">
         <v>0</v>
@@ -9506,7 +9497,7 @@
         <v>216</v>
       </c>
       <c r="B17" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C17" t="s">
         <v>293</v>
@@ -9553,7 +9544,7 @@
         <v>218</v>
       </c>
       <c r="B18" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C18" t="s">
         <v>294</v>
@@ -9568,13 +9559,13 @@
         <v>1836</v>
       </c>
       <c r="G18" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H18">
         <v>250000</v>
       </c>
       <c r="I18" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="J18">
         <v>89.59999999999999</v>
@@ -9600,7 +9591,7 @@
         <v>225</v>
       </c>
       <c r="B19" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C19" t="s">
         <v>295</v>
@@ -9615,7 +9606,7 @@
         <v>1396</v>
       </c>
       <c r="G19" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H19">
         <v>500000</v>
@@ -9753,13 +9744,13 @@
         <v>1124</v>
       </c>
       <c r="G22" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H22">
         <v>0</v>
       </c>
       <c r="I22" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J22">
         <v>88.7</v>
@@ -9785,7 +9776,7 @@
         <v>222</v>
       </c>
       <c r="B23" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C23" t="s">
         <v>299</v>
@@ -9800,7 +9791,7 @@
         <v>1595</v>
       </c>
       <c r="G23" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H23">
         <v>375000</v>
@@ -9832,7 +9823,7 @@
         <v>218</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C24" t="s">
         <v>300</v>
@@ -9847,7 +9838,7 @@
         <v>2016</v>
       </c>
       <c r="G24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H24">
         <v>350000</v>
@@ -9876,10 +9867,10 @@
     </row>
     <row r="25" spans="1:15">
       <c r="A25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B25" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C25" t="s">
         <v>301</v>
@@ -9923,7 +9914,7 @@
         <v>220</v>
       </c>
       <c r="B26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C26" t="s">
         <v>302</v>
@@ -9938,7 +9929,7 @@
         <v>2209</v>
       </c>
       <c r="G26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H26">
         <v>400000</v>
@@ -10030,7 +10021,7 @@
         <v>328</v>
       </c>
       <c r="B2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C2" t="s">
         <v>341</v>
@@ -10045,13 +10036,13 @@
         <v>1382</v>
       </c>
       <c r="G2" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H2">
         <v>2000000</v>
       </c>
       <c r="I2" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J2">
         <v>95.2</v>
@@ -10095,13 +10086,13 @@
         <v>1326</v>
       </c>
       <c r="G3" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H3">
         <v>0</v>
       </c>
       <c r="I3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J3">
         <v>95.09999999999999</v>
@@ -10130,7 +10121,7 @@
         <v>330</v>
       </c>
       <c r="B4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C4" t="s">
         <v>343</v>
@@ -10145,7 +10136,7 @@
         <v>3548</v>
       </c>
       <c r="G4" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H4">
         <v>0</v>
@@ -10198,7 +10189,7 @@
         <v>0</v>
       </c>
       <c r="I5" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J5">
         <v>93.90000000000001</v>
@@ -10277,7 +10268,7 @@
         <v>332</v>
       </c>
       <c r="B7" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C7" t="s">
         <v>346</v>
@@ -10298,7 +10289,7 @@
         <v>1000000</v>
       </c>
       <c r="I7" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J7">
         <v>93.59999999999999</v>
@@ -10348,7 +10339,7 @@
         <v>0</v>
       </c>
       <c r="I8" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="J8">
         <v>93.5</v>
@@ -10377,7 +10368,7 @@
         <v>333</v>
       </c>
       <c r="B9" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C9" t="s">
         <v>348</v>
@@ -10392,13 +10383,13 @@
         <v>1683</v>
       </c>
       <c r="G9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H9">
         <v>0</v>
       </c>
       <c r="I9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J9">
         <v>92.90000000000001</v>
@@ -10495,7 +10486,7 @@
         <v>500000</v>
       </c>
       <c r="I11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J11">
         <v>92.59999999999999</v>
@@ -10539,13 +10530,13 @@
         <v>2019</v>
       </c>
       <c r="G12" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H12">
         <v>800000</v>
       </c>
       <c r="I12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J12">
         <v>92.5</v>
@@ -10589,13 +10580,13 @@
         <v>1483</v>
       </c>
       <c r="G13" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H13">
         <v>350000</v>
       </c>
       <c r="I13" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J13">
         <v>92.5</v>
@@ -10639,7 +10630,7 @@
         <v>1295</v>
       </c>
       <c r="G14" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -10689,13 +10680,13 @@
         <v>2691</v>
       </c>
       <c r="G15" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H15">
         <v>0</v>
       </c>
       <c r="I15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J15">
         <v>91.8</v>
@@ -10739,13 +10730,13 @@
         <v>1202</v>
       </c>
       <c r="G16" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H16">
         <v>0</v>
       </c>
       <c r="I16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J16">
         <v>91.7</v>
@@ -10792,7 +10783,7 @@
         <v>175000</v>
       </c>
       <c r="I17" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J17">
         <v>91.7</v>
@@ -10821,7 +10812,7 @@
         <v>337</v>
       </c>
       <c r="B18" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C18" t="s">
         <v>357</v>
@@ -10836,13 +10827,13 @@
         <v>1367</v>
       </c>
       <c r="G18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H18">
         <v>1400000</v>
       </c>
       <c r="I18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J18">
         <v>91.5</v>
@@ -10989,7 +10980,7 @@
         <v>0</v>
       </c>
       <c r="I21" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J21">
         <v>91</v>
@@ -11089,7 +11080,7 @@
         <v>0</v>
       </c>
       <c r="I23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J23">
         <v>90.40000000000001</v>
@@ -11168,7 +11159,7 @@
         <v>334</v>
       </c>
       <c r="B25" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C25" t="s">
         <v>364</v>
@@ -11302,22 +11293,22 @@
         <v>8</v>
       </c>
       <c r="J1" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="K1" s="1" t="s">
         <v>87</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="L1" s="1" t="s">
         <v>88</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="M1" s="1" t="s">
         <v>89</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="N1" s="1" t="s">
         <v>90</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>91</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:15">
@@ -11393,7 +11384,7 @@
         <v>300000</v>
       </c>
       <c r="I3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J3">
         <v>94.09999999999999</v>
@@ -11440,7 +11431,7 @@
         <v>0</v>
       </c>
       <c r="I4" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J4">
         <v>93.7</v>
@@ -11466,7 +11457,7 @@
         <v>394</v>
       </c>
       <c r="B5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C5" t="s">
         <v>401</v>
@@ -11513,7 +11504,7 @@
         <v>395</v>
       </c>
       <c r="B6" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C6" t="s">
         <v>402</v>
@@ -11560,7 +11551,7 @@
         <v>330</v>
       </c>
       <c r="B7" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C7" t="s">
         <v>403</v>
@@ -11575,7 +11566,7 @@
         <v>1947</v>
       </c>
       <c r="G7" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="H7">
         <v>1000000</v>
@@ -11607,7 +11598,7 @@
         <v>396</v>
       </c>
       <c r="B8" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C8" t="s">
         <v>404</v>
@@ -11625,7 +11616,7 @@
         <v>200000</v>
       </c>
       <c r="I8" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J8">
         <v>91.09999999999999</v>
@@ -11651,7 +11642,7 @@
         <v>397</v>
       </c>
       <c r="B9" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C9" t="s">
         <v>405</v>
@@ -11666,13 +11657,13 @@
         <v>1172</v>
       </c>
       <c r="G9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H9">
         <v>100000</v>
       </c>
       <c r="I9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J9">
         <v>90.8</v>
@@ -11698,7 +11689,7 @@
         <v>330</v>
       </c>
       <c r="B10" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C10" t="s">
         <v>406</v>
@@ -11713,13 +11704,13 @@
         <v>2833</v>
       </c>
       <c r="G10" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H10">
         <v>0</v>
       </c>
       <c r="I10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J10">
         <v>90.7</v>
@@ -11745,7 +11736,7 @@
         <v>329</v>
       </c>
       <c r="B11" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C11" t="s">
         <v>407</v>
@@ -11763,7 +11754,7 @@
         <v>200000</v>
       </c>
       <c r="I11" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J11">
         <v>90.2</v>
@@ -11789,7 +11780,7 @@
         <v>397</v>
       </c>
       <c r="B12" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C12" t="s">
         <v>408</v>
@@ -11810,7 +11801,7 @@
         <v>0</v>
       </c>
       <c r="I12" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J12">
         <v>89.40000000000001</v>
@@ -11883,7 +11874,7 @@
         <v>328</v>
       </c>
       <c r="B14" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C14" t="s">
         <v>410</v>
@@ -11898,13 +11889,13 @@
         <v>3835</v>
       </c>
       <c r="G14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H14">
         <v>800000</v>
       </c>
       <c r="I14" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="J14">
         <v>88.3</v>
@@ -11930,7 +11921,7 @@
         <v>335</v>
       </c>
       <c r="B15" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C15" t="s">
         <v>411</v>
@@ -11948,7 +11939,7 @@
         <v>175000</v>
       </c>
       <c r="I15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J15">
         <v>88.2</v>
@@ -11992,7 +11983,7 @@
         <v>850000</v>
       </c>
       <c r="I16" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J16">
         <v>87.8</v>
@@ -12033,13 +12024,13 @@
         <v>1324</v>
       </c>
       <c r="G17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H17">
         <v>850000</v>
       </c>
       <c r="I17" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J17">
         <v>87.40000000000001</v>
@@ -12065,7 +12056,7 @@
         <v>395</v>
       </c>
       <c r="B18" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C18" t="s">
         <v>346</v>
@@ -12086,7 +12077,7 @@
         <v>250000</v>
       </c>
       <c r="I18" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J18">
         <v>87.2</v>
@@ -12174,13 +12165,13 @@
         <v>1732</v>
       </c>
       <c r="G20" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="H20">
         <v>0</v>
       </c>
       <c r="I20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J20">
         <v>86.59999999999999</v>
@@ -12206,7 +12197,7 @@
         <v>333</v>
       </c>
       <c r="B21" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C21" t="s">
         <v>416</v>
@@ -12221,7 +12212,7 @@
         <v>1395</v>
       </c>
       <c r="G21" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H21">
         <v>450000</v>
@@ -12253,7 +12244,7 @@
         <v>337</v>
       </c>
       <c r="B22" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C22" t="s">
         <v>417</v>
@@ -12271,7 +12262,7 @@
         <v>400000</v>
       </c>
       <c r="I22" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J22">
         <v>85.2</v>
@@ -12312,13 +12303,13 @@
         <v>1486</v>
       </c>
       <c r="G23" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="H23">
         <v>0</v>
       </c>
       <c r="I23" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J23">
         <v>85.2</v>
@@ -12344,7 +12335,7 @@
         <v>337</v>
       </c>
       <c r="B24" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C24" t="s">
         <v>419</v>
@@ -12359,13 +12350,13 @@
         <v>1533</v>
       </c>
       <c r="G24" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="H24">
         <v>1200000</v>
       </c>
       <c r="I24" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J24">
         <v>85.09999999999999</v>
@@ -12438,7 +12429,7 @@
         <v>332</v>
       </c>
       <c r="B26" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C26" t="s">
         <v>421</v>
@@ -12459,7 +12450,7 @@
         <v>400000</v>
       </c>
       <c r="I26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="J26">
         <v>84.90000000000001</v>

</xml_diff>

<commit_message>
Rodinei fora das listas (contratado pelo Santos)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EuPBN7B2QoMn8WDwKax4KN
</commit_message>
<xml_diff>
--- a/Santa Cruz V2/listas/bola_parada_especialistas.xlsx
+++ b/Santa Cruz V2/listas/bola_parada_especialistas.xlsx
@@ -1073,12 +1073,12 @@
     <t>Evander</t>
   </si>
   <si>
+    <t>J. Bartolo</t>
+  </si>
+  <si>
     <t>Arthur Rezende</t>
   </si>
   <si>
-    <t>J. Bartolo</t>
-  </si>
-  <si>
     <t>Valdívia</t>
   </si>
   <si>
@@ -1148,10 +1148,10 @@
     <t>Cincinnati</t>
   </si>
   <si>
+    <t>Asteras Tripolis</t>
+  </si>
+  <si>
     <t>Muharraq</t>
-  </si>
-  <si>
-    <t>Asteras Tripolis</t>
   </si>
   <si>
     <t>Jeonnam Dragons</t>
@@ -10421,10 +10421,10 @@
     </row>
     <row r="10" spans="1:16">
       <c r="A10" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B10" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C10" t="s">
         <v>350</v>
@@ -10433,45 +10433,48 @@
         <v>375</v>
       </c>
       <c r="E10">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="F10">
-        <v>1839</v>
+        <v>2529</v>
+      </c>
+      <c r="G10" t="s">
+        <v>390</v>
       </c>
       <c r="H10">
-        <v>500000</v>
+        <v>600000</v>
       </c>
       <c r="I10" t="s">
-        <v>81</v>
+        <v>179</v>
       </c>
       <c r="J10">
         <v>92.59999999999999</v>
       </c>
       <c r="K10">
-        <v>56</v>
+        <v>104</v>
       </c>
       <c r="L10">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="M10">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="N10">
-        <v>22.2</v>
+        <v>37.5</v>
       </c>
       <c r="O10">
-        <v>0.16</v>
+        <v>0.21</v>
       </c>
       <c r="P10">
-        <v>38.1</v>
+        <v>28.6</v>
       </c>
     </row>
     <row r="11" spans="1:16">
       <c r="A11" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="B11" t="s">
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C11" t="s">
         <v>351</v>
@@ -10480,40 +10483,37 @@
         <v>376</v>
       </c>
       <c r="E11">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="F11">
-        <v>2529</v>
-      </c>
-      <c r="G11" t="s">
-        <v>390</v>
+        <v>1839</v>
       </c>
       <c r="H11">
-        <v>600000</v>
+        <v>500000</v>
       </c>
       <c r="I11" t="s">
-        <v>179</v>
+        <v>81</v>
       </c>
       <c r="J11">
         <v>92.59999999999999</v>
       </c>
       <c r="K11">
-        <v>104</v>
+        <v>56</v>
       </c>
       <c r="L11">
-        <v>52</v>
+        <v>24</v>
       </c>
       <c r="M11">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N11">
-        <v>37.5</v>
+        <v>22.2</v>
       </c>
       <c r="O11">
-        <v>0.21</v>
+        <v>0.16</v>
       </c>
       <c r="P11">
-        <v>28.6</v>
+        <v>38.1</v>
       </c>
     </row>
     <row r="12" spans="1:16">

</xml_diff>